<commit_message>
Admin: edit data/shala-calendar.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/shala-calendar.xlsx
+++ b/data/shala-calendar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G74"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -867,19 +867,19 @@
         <v>December</v>
       </c>
       <c r="C21" t="str">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D21" t="str">
-        <v>Marathi Shala</v>
+        <v>Midterm Exam</v>
       </c>
       <c r="E21" t="str">
-        <v>Class</v>
+        <v>Exam</v>
       </c>
       <c r="F21" t="str">
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>Online · Week 16</v>
+        <v>In-person</v>
       </c>
     </row>
     <row r="22">
@@ -890,42 +890,42 @@
         <v>December</v>
       </c>
       <c r="C22" t="str">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D22" t="str">
-        <v>Marathi Shala</v>
+        <v>Midterm Exam</v>
       </c>
       <c r="E22" t="str">
-        <v>Class</v>
+        <v>Exam</v>
       </c>
       <c r="F22" t="str">
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>Online · Week 17</v>
+        <v>In-person</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B23" t="str">
-        <v>January</v>
+        <v>December</v>
       </c>
       <c r="C23" t="str">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D23" t="str">
-        <v>Midterm Exam</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E23" t="str">
-        <v>Exam</v>
+        <v>Class</v>
       </c>
       <c r="F23" t="str">
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>In-person</v>
+        <v>Online · Week 16</v>
       </c>
     </row>
     <row r="24">
@@ -936,19 +936,19 @@
         <v>December</v>
       </c>
       <c r="C24" t="str">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D24" t="str">
-        <v>Marathi Shala</v>
+        <v>Midterm Exam</v>
       </c>
       <c r="E24" t="str">
-        <v>Class</v>
+        <v>Exam</v>
       </c>
       <c r="F24" t="str">
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>Online · Week 17</v>
+        <v>In-person</v>
       </c>
     </row>
     <row r="25">
@@ -959,19 +959,19 @@
         <v>December</v>
       </c>
       <c r="C25" t="str">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D25" t="str">
-        <v>Christmas &amp; New Year Break</v>
+        <v>Midterm Exam</v>
       </c>
       <c r="E25" t="str">
-        <v>Holiday</v>
+        <v>Exam</v>
       </c>
       <c r="F25" t="str">
         <v/>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>In-person</v>
       </c>
     </row>
     <row r="26">
@@ -982,19 +982,19 @@
         <v>December</v>
       </c>
       <c r="C26" t="str">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D26" t="str">
-        <v>Christmas &amp; New Year Break</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E26" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F26" t="str">
         <v/>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>Online · Week 17</v>
       </c>
     </row>
     <row r="27">
@@ -1005,7 +1005,7 @@
         <v>December</v>
       </c>
       <c r="C27" t="str">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D27" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1028,7 +1028,7 @@
         <v>December</v>
       </c>
       <c r="C28" t="str">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D28" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1051,7 +1051,7 @@
         <v>December</v>
       </c>
       <c r="C29" t="str">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D29" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1074,7 +1074,7 @@
         <v>December</v>
       </c>
       <c r="C30" t="str">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D30" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1097,7 +1097,7 @@
         <v>December</v>
       </c>
       <c r="C31" t="str">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D31" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1120,7 +1120,7 @@
         <v>December</v>
       </c>
       <c r="C32" t="str">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D32" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B33" t="str">
-        <v>January</v>
+        <v>December</v>
       </c>
       <c r="C33" t="str">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D33" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1160,13 +1160,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B34" t="str">
-        <v>January</v>
+        <v>December</v>
       </c>
       <c r="C34" t="str">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D34" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1189,7 +1189,7 @@
         <v>January</v>
       </c>
       <c r="C35" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" t="str">
         <v>Christmas &amp; New Year Break</v>
@@ -1212,19 +1212,19 @@
         <v>January</v>
       </c>
       <c r="C36" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D36" t="str">
-        <v>Marathi Shala</v>
+        <v>Christmas &amp; New Year Break</v>
       </c>
       <c r="E36" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F36" t="str">
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>Online · Week 18</v>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1235,19 +1235,19 @@
         <v>January</v>
       </c>
       <c r="C37" t="str">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D37" t="str">
-        <v>Marathi Shala</v>
+        <v>Christmas &amp; New Year Break</v>
       </c>
       <c r="E37" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F37" t="str">
         <v/>
       </c>
       <c r="G37" t="str">
-        <v>Online · Week 19</v>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1258,19 +1258,19 @@
         <v>January</v>
       </c>
       <c r="C38" t="str">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D38" t="str">
-        <v>MLK Day</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E38" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F38" t="str">
         <v/>
       </c>
       <c r="G38" t="str">
-        <v/>
+        <v>Online · Week 18</v>
       </c>
     </row>
     <row r="39">
@@ -1281,7 +1281,7 @@
         <v>January</v>
       </c>
       <c r="C39" t="str">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D39" t="str">
         <v>Marathi Shala</v>
@@ -1293,7 +1293,7 @@
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>Online · Week 20</v>
+        <v>Online · Week 19</v>
       </c>
     </row>
     <row r="40">
@@ -1304,19 +1304,19 @@
         <v>January</v>
       </c>
       <c r="C40" t="str">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D40" t="str">
-        <v>Marathi Shala</v>
+        <v>MLK Day</v>
       </c>
       <c r="E40" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F40" t="str">
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>Online · Week 21</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -1324,10 +1324,10 @@
         <v>2027</v>
       </c>
       <c r="B41" t="str">
-        <v>February</v>
+        <v>January</v>
       </c>
       <c r="C41" t="str">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D41" t="str">
         <v>Marathi Shala</v>
@@ -1339,7 +1339,7 @@
         <v/>
       </c>
       <c r="G41" t="str">
-        <v>Online · Week 22</v>
+        <v>Online · Week 20</v>
       </c>
     </row>
     <row r="42">
@@ -1347,10 +1347,10 @@
         <v>2027</v>
       </c>
       <c r="B42" t="str">
-        <v>February</v>
+        <v>January</v>
       </c>
       <c r="C42" t="str">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D42" t="str">
         <v>Marathi Shala</v>
@@ -1362,7 +1362,7 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>Online · Week 23</v>
+        <v>Online · Week 21</v>
       </c>
     </row>
     <row r="43">
@@ -1373,19 +1373,19 @@
         <v>February</v>
       </c>
       <c r="C43" t="str">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D43" t="str">
-        <v>Winter Break</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E43" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F43" t="str">
         <v/>
       </c>
       <c r="G43" t="str">
-        <v/>
+        <v>Online · Week 22</v>
       </c>
     </row>
     <row r="44">
@@ -1396,19 +1396,19 @@
         <v>February</v>
       </c>
       <c r="C44" t="str">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D44" t="str">
-        <v>Winter Break</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E44" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F44" t="str">
         <v/>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Online · Week 23</v>
       </c>
     </row>
     <row r="45">
@@ -1419,7 +1419,7 @@
         <v>February</v>
       </c>
       <c r="C45" t="str">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D45" t="str">
         <v>Winter Break</v>
@@ -1442,7 +1442,7 @@
         <v>February</v>
       </c>
       <c r="C46" t="str">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D46" t="str">
         <v>Winter Break</v>
@@ -1465,7 +1465,7 @@
         <v>February</v>
       </c>
       <c r="C47" t="str">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D47" t="str">
         <v>Winter Break</v>
@@ -1488,19 +1488,19 @@
         <v>February</v>
       </c>
       <c r="C48" t="str">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D48" t="str">
-        <v>Marathi Shala</v>
+        <v>Winter Break</v>
       </c>
       <c r="E48" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F48" t="str">
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>Online · Week 24</v>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -1508,22 +1508,22 @@
         <v>2027</v>
       </c>
       <c r="B49" t="str">
-        <v>March</v>
+        <v>February</v>
       </c>
       <c r="C49" t="str">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D49" t="str">
-        <v>Marathi Shala</v>
+        <v>Winter Break</v>
       </c>
       <c r="E49" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F49" t="str">
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>Online · Week 25</v>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -1531,10 +1531,10 @@
         <v>2027</v>
       </c>
       <c r="B50" t="str">
-        <v>March</v>
+        <v>February</v>
       </c>
       <c r="C50" t="str">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D50" t="str">
         <v>Marathi Shala</v>
@@ -1546,7 +1546,7 @@
         <v/>
       </c>
       <c r="G50" t="str">
-        <v>Online · Week 26</v>
+        <v>Online · Week 24</v>
       </c>
     </row>
     <row r="51">
@@ -1557,7 +1557,7 @@
         <v>March</v>
       </c>
       <c r="C51" t="str">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D51" t="str">
         <v>Marathi Shala</v>
@@ -1569,7 +1569,7 @@
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>Online · Week 27</v>
+        <v>Online · Week 25</v>
       </c>
     </row>
     <row r="52">
@@ -1580,7 +1580,7 @@
         <v>March</v>
       </c>
       <c r="C52" t="str">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D52" t="str">
         <v>Marathi Shala</v>
@@ -1592,7 +1592,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>Online · Week 28</v>
+        <v>Online · Week 26</v>
       </c>
     </row>
     <row r="53">
@@ -1603,19 +1603,19 @@
         <v>March</v>
       </c>
       <c r="C53" t="str">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D53" t="str">
-        <v>Good Friday</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E53" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F53" t="str">
         <v/>
       </c>
       <c r="G53" t="str">
-        <v/>
+        <v>Online · Week 27</v>
       </c>
     </row>
     <row r="54">
@@ -1626,7 +1626,7 @@
         <v>March</v>
       </c>
       <c r="C54" t="str">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D54" t="str">
         <v>Marathi Shala</v>
@@ -1638,7 +1638,7 @@
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>Online · Week 29</v>
+        <v>Online · Week 28</v>
       </c>
     </row>
     <row r="55">
@@ -1646,22 +1646,22 @@
         <v>2027</v>
       </c>
       <c r="B55" t="str">
-        <v>April</v>
+        <v>March</v>
       </c>
       <c r="C55" t="str">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="D55" t="str">
-        <v>Marathi Shala</v>
+        <v>Good Friday</v>
       </c>
       <c r="E55" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F55" t="str">
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>Online · Week 30</v>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -1669,22 +1669,22 @@
         <v>2027</v>
       </c>
       <c r="B56" t="str">
-        <v>April</v>
+        <v>March</v>
       </c>
       <c r="C56" t="str">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="D56" t="str">
-        <v>Gudhi Padwa</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E56" t="str">
-        <v>Event</v>
+        <v>Class</v>
       </c>
       <c r="F56" t="str">
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>In-person</v>
+        <v>Online · Week 29</v>
       </c>
     </row>
     <row r="57">
@@ -1695,7 +1695,7 @@
         <v>April</v>
       </c>
       <c r="C57" t="str">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D57" t="str">
         <v>Marathi Shala</v>
@@ -1707,7 +1707,7 @@
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>Online · Week 31</v>
+        <v>Online · Week 30</v>
       </c>
     </row>
     <row r="58">
@@ -1718,19 +1718,19 @@
         <v>April</v>
       </c>
       <c r="C58" t="str">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D58" t="str">
-        <v>Spring Break</v>
+        <v>Gudhi Padwa</v>
       </c>
       <c r="E58" t="str">
-        <v>Holiday</v>
+        <v>Event</v>
       </c>
       <c r="F58" t="str">
         <v/>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>In-person</v>
       </c>
     </row>
     <row r="59">
@@ -1741,19 +1741,19 @@
         <v>April</v>
       </c>
       <c r="C59" t="str">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D59" t="str">
-        <v>Spring Break</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E59" t="str">
-        <v>Holiday</v>
+        <v>Class</v>
       </c>
       <c r="F59" t="str">
         <v/>
       </c>
       <c r="G59" t="str">
-        <v/>
+        <v>Online · Week 31</v>
       </c>
     </row>
     <row r="60">
@@ -1764,7 +1764,7 @@
         <v>April</v>
       </c>
       <c r="C60" t="str">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D60" t="str">
         <v>Spring Break</v>
@@ -1787,7 +1787,7 @@
         <v>April</v>
       </c>
       <c r="C61" t="str">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D61" t="str">
         <v>Spring Break</v>
@@ -1810,7 +1810,7 @@
         <v>April</v>
       </c>
       <c r="C62" t="str">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D62" t="str">
         <v>Spring Break</v>
@@ -1833,19 +1833,19 @@
         <v>April</v>
       </c>
       <c r="C63" t="str">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D63" t="str">
-        <v>Marathi Shala</v>
+        <v>Spring Break</v>
       </c>
       <c r="E63" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F63" t="str">
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>Online · Week 32</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -1853,22 +1853,22 @@
         <v>2027</v>
       </c>
       <c r="B64" t="str">
-        <v>May</v>
+        <v>April</v>
       </c>
       <c r="C64" t="str">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="D64" t="str">
-        <v>Marathi Shala</v>
+        <v>Spring Break</v>
       </c>
       <c r="E64" t="str">
-        <v>Class</v>
+        <v>Holiday</v>
       </c>
       <c r="F64" t="str">
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>Online · Week 33</v>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -1876,10 +1876,10 @@
         <v>2027</v>
       </c>
       <c r="B65" t="str">
-        <v>May</v>
+        <v>April</v>
       </c>
       <c r="C65" t="str">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D65" t="str">
         <v>Marathi Shala</v>
@@ -1891,7 +1891,7 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>Online · Week 34</v>
+        <v>Online · Week 32</v>
       </c>
     </row>
     <row r="66">
@@ -1902,19 +1902,19 @@
         <v>May</v>
       </c>
       <c r="C66" t="str">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D66" t="str">
-        <v>Final Exam</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E66" t="str">
-        <v>Exam</v>
+        <v>Class</v>
       </c>
       <c r="F66" t="str">
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>In-person</v>
+        <v>Online · Week 33</v>
       </c>
     </row>
     <row r="67">
@@ -1925,19 +1925,19 @@
         <v>May</v>
       </c>
       <c r="C67" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D67" t="str">
-        <v>Final Exam</v>
+        <v>Marathi Shala</v>
       </c>
       <c r="E67" t="str">
-        <v>Exam</v>
+        <v>Class</v>
       </c>
       <c r="F67" t="str">
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>In-person</v>
+        <v>Online · Week 34</v>
       </c>
     </row>
     <row r="68">
@@ -1948,7 +1948,7 @@
         <v>May</v>
       </c>
       <c r="C68" t="str">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D68" t="str">
         <v>Final Exam</v>
@@ -1971,7 +1971,7 @@
         <v>May</v>
       </c>
       <c r="C69" t="str">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D69" t="str">
         <v>Final Exam</v>
@@ -1991,16 +1991,16 @@
         <v>2027</v>
       </c>
       <c r="B70" t="str">
-        <v>June</v>
+        <v>May</v>
       </c>
       <c r="C70" t="str">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D70" t="str">
-        <v>Picnic</v>
+        <v>Final Exam</v>
       </c>
       <c r="E70" t="str">
-        <v>Event</v>
+        <v>Exam</v>
       </c>
       <c r="F70" t="str">
         <v/>
@@ -2014,16 +2014,16 @@
         <v>2027</v>
       </c>
       <c r="B71" t="str">
-        <v>June</v>
+        <v>May</v>
       </c>
       <c r="C71" t="str">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D71" t="str">
-        <v>Picnic (rain date)</v>
+        <v>Final Exam</v>
       </c>
       <c r="E71" t="str">
-        <v>Event</v>
+        <v>Exam</v>
       </c>
       <c r="F71" t="str">
         <v/>
@@ -2034,16 +2034,16 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="B72" t="str">
-        <v>Nov</v>
+        <v>June</v>
       </c>
       <c r="C72" t="str">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D72" t="str">
-        <v>Diwali Activity</v>
+        <v>Picnic</v>
       </c>
       <c r="E72" t="str">
         <v>Event</v>
@@ -2055,9 +2055,55 @@
         <v>In-person</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>2027</v>
+      </c>
+      <c r="B73" t="str">
+        <v>June</v>
+      </c>
+      <c r="C73" t="str">
+        <v>13</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Picnic (rain date)</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Event</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v>In-person</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>2026</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Nov</v>
+      </c>
+      <c r="C74" t="str">
+        <v>15</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Diwali Activity</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Event</v>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+      <c r="G74" t="str">
+        <v>In-person</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G74"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>